<commit_message>
statuto degli Imported generato dall'ETL (B2, D-068)
258 letture S-auto-{luogo} con atto (Lorenzo, ReferentialEvidence,
adottate, validate, data costante); fonte del repertorio dall'owl:sameAs
esterno dell'ancora (oggi 0 su 258). IQ13 su tutti i 309 luoghi;
StatusRationaleShape su tutti i luoghi (avvertenze 48 -> 50). C2:
descrizione di castello.
ABox 32.385 -> 38.588.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Sources.xlsx
+++ b/data/source/xlsx/Sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -700,6 +700,65 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>wikidata</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wikidata</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Wikidata, base di conoscenza libera (Wikimedia Foundation). https://www.wikidata.org</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Wikimedia Foundation</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>repertorio</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Repertorio di un identificatore esterno (owl:sameAs) dell'ancora; usato dalle letture di statuto generate (D-068).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>geonames</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>GeoNames</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GeoNames, base di dati geografica. https://www.geonames.org</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>repertorio</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Come sopra (D-068).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>